<commit_message>
Add create admin superuser command for production
</commit_message>
<xml_diff>
--- a/static/templates/plantilla_estudiantes.xlsx
+++ b/static/templates/plantilla_estudiantes.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Estudiantes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +31,14 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002196F3"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -40,12 +49,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="004CAF50"/>
+        <bgColor rgb="004CAF50"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -53,24 +62,17 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,91 +438,199 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Teléfono</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Nombre</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Teléfono</t>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cédula</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Juan Pérez</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>573001234567</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>María García</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>📚 PLANTILLA DE IMPORTACIÓN DE ESTUDIANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>María García</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>573009876543</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Columnas requeridas:</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Carlos López</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>573005555555</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Ana Martínez</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>573004444444</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Columna A - Teléfono:</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Número de WhatsApp con código de país (ej: 573001234567)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Pedro Rodríguez</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>573003333333</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Columna B - Nombre:</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Nombre completo del estudiante</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Columna C - Cédula:</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Número de cédula SIN puntos ni espacios (ej: 1234567890)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ IMPORTANTE:</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>• La cédula es el identificador único de cada estudiante</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>• No puede haber dos estudiantes con la misma cédula</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>• Si la cédula ya existe, se actualizarán los datos</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>• El teléfono debe incluir código de país (57 para Colombia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>• Todos los campos son obligatorios</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Ejemplo de datos válidos:</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Teléfono: 573001234567</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Nombre: María García</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cédula: 1234567890</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Error de Validación" error="El teléfono debe ser un número" type="custom">
-      <formula1>=NOT(ISERROR(VALUE(B2:B1000)))</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>